<commit_message>
Add source links to requirements
</commit_message>
<xml_diff>
--- a/jm-test/Minime_Mode_Test_Cases.xlsx
+++ b/jm-test/Minime_Mode_Test_Cases.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="9060"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements" sheetId="5" r:id="rId1"/>
@@ -70,10 +70,10 @@
     <t>Minime Mode is minimized to a corner of the screen.</t>
   </si>
   <si>
-    <t>Minime Mode documentation.</t>
-  </si>
-  <si>
-    <t>Documentation-derived</t>
+    <t>Official Minime Mode documentation included in Assignment brief</t>
+  </si>
+  <si>
+    <t>Documentation</t>
   </si>
   <si>
     <t>MM-003</t>
@@ -1365,18 +1365,18 @@
       <charset val="0"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1855,28 +1855,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2000,7 +2000,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2039,6 +2039,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2582,7 +2585,7 @@
       <c r="B3" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="14" t="s">
         <v>12</v>
       </c>
       <c r="D3" s="13" t="s">
@@ -2599,7 +2602,7 @@
       <c r="B4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="13" t="s">
@@ -2616,7 +2619,7 @@
       <c r="B5" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="13" t="s">
@@ -3120,6 +3123,11 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C3" r:id="rId1" display="Official Minime Mode documentation included in Assignment brief"/>
+    <hyperlink ref="C4" r:id="rId1" display="Official Minime Mode documentation included in Assignment brief"/>
+    <hyperlink ref="C5" r:id="rId1" display="Official Minime Mode documentation included in Assignment brief"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>